<commit_message>
chore(reports): refresh generated execution reports
Regenerated by the runs made while verifying this branch. Tracked here by
convention, as in d73d1d6 and 7a8d1c0.

Co-Authored-By: Claude Opus 5 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/reports/Test-Cases.xlsx
+++ b/reports/Test-Cases.xlsx
@@ -16,7 +16,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="644" uniqueCount="360">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="644" uniqueCount="357">
   <si>
     <t>FEATURE</t>
   </si>
@@ -64,12 +64,6 @@
   </si>
   <si>
     <t>Order-01</t>
-  </si>
-  <si>
-    <t>2026-07-16 18:15:17</t>
-  </si>
-  <si>
-    <t>FAIL</t>
   </si>
   <si>
     <t>user-signup</t>
@@ -586,9 +580,6 @@
     <t>5 new 'Submitted' vendor orders exist in /order-history</t>
   </si>
   <si>
-    <t>Failed in 44.9s: Error: AC (order details): expected "Sprite" in the opened order details (order opened = "PFG — 07/16/2026"). Note: exploration found "Sprite" in the SYSCO order; a freshly-sent batch's list order is non-deterministic, so "order number 2" is not a stable reference to the Sprite-containing order.</t>
-  </si>
-  <si>
     <t>SignUp-001-AC1-POS-01</t>
   </si>
   <si>
@@ -1207,7 +1198,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
-  <fonts count="7" x14ac:knownFonts="1">
+  <fonts count="6" x14ac:knownFonts="1">
     <font>
       <color theme="1"/>
       <family val="2"/>
@@ -1233,12 +1224,6 @@
     </font>
     <font>
       <b/>
-      <color rgb="FF721C24"/>
-      <sz val="10.5"/>
-      <name val="Calibri"/>
-    </font>
-    <font>
-      <b/>
       <sz val="11"/>
       <name val="Calibri"/>
     </font>
@@ -1249,7 +1234,7 @@
       <name val="Calibri"/>
     </font>
   </fonts>
-  <fills count="7">
+  <fills count="6">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -1264,11 +1249,6 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="FFFFF3CD"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFF8D7DA"/>
       </patternFill>
     </fill>
     <fill>
@@ -1309,7 +1289,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="7">
+  <cellXfs count="6">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -1321,12 +1301,9 @@
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="6" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -1763,24 +1740,24 @@
         <v>0</v>
       </c>
       <c r="G3" s="2">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="H3" s="2">
         <v>0</v>
       </c>
       <c r="I3" s="2" t="s">
-        <v>16</v>
-      </c>
-      <c r="J3" s="4" t="s">
-        <v>17</v>
+        <v>12</v>
+      </c>
+      <c r="J3" s="3" t="s">
+        <v>13</v>
       </c>
     </row>
     <row r="4" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A4" s="2" t="s">
-        <v>18</v>
+        <v>16</v>
       </c>
       <c r="B4" s="2" t="s">
-        <v>19</v>
+        <v>17</v>
       </c>
       <c r="C4" s="2">
         <v>26</v>
@@ -1809,10 +1786,10 @@
     </row>
     <row r="5" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A5" s="2" t="s">
-        <v>20</v>
+        <v>18</v>
       </c>
       <c r="B5" s="2" t="s">
-        <v>21</v>
+        <v>19</v>
       </c>
       <c r="C5" s="2">
         <v>3</v>
@@ -1841,10 +1818,10 @@
     </row>
     <row r="6" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A6" s="2" t="s">
-        <v>22</v>
+        <v>20</v>
       </c>
       <c r="B6" s="2" t="s">
-        <v>23</v>
+        <v>21</v>
       </c>
       <c r="C6" s="2">
         <v>4</v>
@@ -1872,35 +1849,35 @@
       </c>
     </row>
     <row r="7" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A7" s="5" t="s">
-        <v>24</v>
-      </c>
-      <c r="B7" s="5" t="s">
-        <v>25</v>
-      </c>
-      <c r="C7" s="5">
+      <c r="A7" s="4" t="s">
+        <v>22</v>
+      </c>
+      <c r="B7" s="4" t="s">
+        <v>23</v>
+      </c>
+      <c r="C7" s="4">
         <v>56</v>
       </c>
-      <c r="D7" s="5">
+      <c r="D7" s="4">
         <v>36</v>
       </c>
-      <c r="E7" s="5">
+      <c r="E7" s="4">
         <v>20</v>
       </c>
-      <c r="F7" s="5">
+      <c r="F7" s="4">
         <v>0</v>
       </c>
-      <c r="G7" s="5">
-        <v>1</v>
-      </c>
-      <c r="H7" s="5">
+      <c r="G7" s="4">
         <v>0</v>
       </c>
-      <c r="I7" s="5" t="s">
-        <v>25</v>
-      </c>
-      <c r="J7" s="5" t="s">
-        <v>25</v>
+      <c r="H7" s="4">
+        <v>0</v>
+      </c>
+      <c r="I7" s="4" t="s">
+        <v>23</v>
+      </c>
+      <c r="J7" s="4" t="s">
+        <v>23</v>
       </c>
     </row>
   </sheetData>
@@ -1928,63 +1905,63 @@
   <sheetData>
     <row r="1" ht="28" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
+        <v>24</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>25</v>
+      </c>
+      <c r="C1" s="1" t="s">
         <v>26</v>
       </c>
-      <c r="B1" s="1" t="s">
+      <c r="D1" s="1" t="s">
         <v>27</v>
       </c>
-      <c r="C1" s="1" t="s">
+      <c r="E1" s="1" t="s">
         <v>28</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="F1" s="1" t="s">
         <v>29</v>
       </c>
-      <c r="E1" s="1" t="s">
+      <c r="G1" s="1" t="s">
         <v>30</v>
       </c>
-      <c r="F1" s="1" t="s">
+      <c r="H1" s="1" t="s">
         <v>31</v>
       </c>
-      <c r="G1" s="1" t="s">
+      <c r="I1" s="1" t="s">
         <v>32</v>
       </c>
-      <c r="H1" s="1" t="s">
+      <c r="J1" s="1" t="s">
         <v>33</v>
-      </c>
-      <c r="I1" s="1" t="s">
-        <v>34</v>
-      </c>
-      <c r="J1" s="1" t="s">
-        <v>35</v>
       </c>
     </row>
     <row r="2" ht="64" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A2" s="2" t="s">
+        <v>34</v>
+      </c>
+      <c r="B2" s="2" t="s">
+        <v>35</v>
+      </c>
+      <c r="C2" s="2" t="s">
         <v>36</v>
       </c>
-      <c r="B2" s="2" t="s">
+      <c r="D2" s="2" t="s">
         <v>37</v>
       </c>
-      <c r="C2" s="2" t="s">
+      <c r="E2" s="2" t="s">
         <v>38</v>
       </c>
-      <c r="D2" s="2" t="s">
+      <c r="F2" s="2" t="s">
         <v>39</v>
       </c>
-      <c r="E2" s="2" t="s">
+      <c r="G2" s="2" t="s">
         <v>40</v>
       </c>
-      <c r="F2" s="2" t="s">
+      <c r="H2" s="2" t="s">
         <v>41</v>
       </c>
-      <c r="G2" s="2" t="s">
+      <c r="I2" s="2" t="s">
         <v>42</v>
-      </c>
-      <c r="H2" s="2" t="s">
-        <v>43</v>
-      </c>
-      <c r="I2" s="2" t="s">
-        <v>44</v>
       </c>
       <c r="J2" s="3" t="s">
         <v>13</v>
@@ -1992,31 +1969,31 @@
     </row>
     <row r="3" ht="48" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A3" s="2" t="s">
+        <v>43</v>
+      </c>
+      <c r="B3" s="2" t="s">
+        <v>44</v>
+      </c>
+      <c r="C3" s="2" t="s">
         <v>45</v>
       </c>
-      <c r="B3" s="2" t="s">
+      <c r="D3" s="2" t="s">
         <v>46</v>
       </c>
-      <c r="C3" s="2" t="s">
+      <c r="E3" s="2" t="s">
         <v>47</v>
       </c>
-      <c r="D3" s="2" t="s">
+      <c r="F3" s="2" t="s">
         <v>48</v>
       </c>
-      <c r="E3" s="2" t="s">
+      <c r="G3" s="2" t="s">
         <v>49</v>
       </c>
-      <c r="F3" s="2" t="s">
+      <c r="H3" s="2" t="s">
         <v>50</v>
       </c>
-      <c r="G3" s="2" t="s">
-        <v>51</v>
-      </c>
-      <c r="H3" s="2" t="s">
-        <v>52</v>
-      </c>
       <c r="I3" s="2" t="s">
-        <v>44</v>
+        <v>42</v>
       </c>
       <c r="J3" s="3" t="s">
         <v>13</v>
@@ -2024,31 +2001,31 @@
     </row>
     <row r="4" ht="48" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A4" s="2" t="s">
+        <v>51</v>
+      </c>
+      <c r="B4" s="2" t="s">
+        <v>52</v>
+      </c>
+      <c r="C4" s="2" t="s">
         <v>53</v>
       </c>
-      <c r="B4" s="2" t="s">
+      <c r="D4" s="2" t="s">
+        <v>46</v>
+      </c>
+      <c r="E4" s="2" t="s">
         <v>54</v>
       </c>
-      <c r="C4" s="2" t="s">
+      <c r="F4" s="2" t="s">
         <v>55</v>
       </c>
-      <c r="D4" s="2" t="s">
-        <v>48</v>
-      </c>
-      <c r="E4" s="2" t="s">
-        <v>56</v>
-      </c>
-      <c r="F4" s="2" t="s">
-        <v>57</v>
-      </c>
       <c r="G4" s="2" t="s">
-        <v>51</v>
+        <v>49</v>
       </c>
       <c r="H4" s="2" t="s">
-        <v>52</v>
+        <v>50</v>
       </c>
       <c r="I4" s="2" t="s">
-        <v>44</v>
+        <v>42</v>
       </c>
       <c r="J4" s="3" t="s">
         <v>13</v>
@@ -2056,31 +2033,31 @@
     </row>
     <row r="5" ht="48" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A5" s="2" t="s">
+        <v>56</v>
+      </c>
+      <c r="B5" s="2" t="s">
+        <v>57</v>
+      </c>
+      <c r="C5" s="2" t="s">
         <v>58</v>
       </c>
-      <c r="B5" s="2" t="s">
+      <c r="D5" s="2" t="s">
+        <v>46</v>
+      </c>
+      <c r="E5" s="2" t="s">
         <v>59</v>
       </c>
-      <c r="C5" s="2" t="s">
+      <c r="F5" s="2" t="s">
         <v>60</v>
       </c>
-      <c r="D5" s="2" t="s">
-        <v>48</v>
-      </c>
-      <c r="E5" s="2" t="s">
+      <c r="G5" s="2" t="s">
         <v>61</v>
       </c>
-      <c r="F5" s="2" t="s">
+      <c r="H5" s="2" t="s">
         <v>62</v>
       </c>
-      <c r="G5" s="2" t="s">
-        <v>63</v>
-      </c>
-      <c r="H5" s="2" t="s">
-        <v>64</v>
-      </c>
       <c r="I5" s="2" t="s">
-        <v>44</v>
+        <v>42</v>
       </c>
       <c r="J5" s="3" t="s">
         <v>13</v>
@@ -2088,31 +2065,31 @@
     </row>
     <row r="6" ht="48" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A6" s="2" t="s">
+        <v>63</v>
+      </c>
+      <c r="B6" s="2" t="s">
+        <v>64</v>
+      </c>
+      <c r="C6" s="2" t="s">
         <v>65</v>
       </c>
-      <c r="B6" s="2" t="s">
+      <c r="D6" s="2" t="s">
+        <v>46</v>
+      </c>
+      <c r="E6" s="2" t="s">
         <v>66</v>
       </c>
-      <c r="C6" s="2" t="s">
+      <c r="F6" s="2" t="s">
         <v>67</v>
       </c>
-      <c r="D6" s="2" t="s">
-        <v>48</v>
-      </c>
-      <c r="E6" s="2" t="s">
-        <v>68</v>
-      </c>
-      <c r="F6" s="2" t="s">
-        <v>69</v>
-      </c>
       <c r="G6" s="2" t="s">
-        <v>63</v>
+        <v>61</v>
       </c>
       <c r="H6" s="2" t="s">
-        <v>64</v>
+        <v>62</v>
       </c>
       <c r="I6" s="2" t="s">
-        <v>44</v>
+        <v>42</v>
       </c>
       <c r="J6" s="3" t="s">
         <v>13</v>
@@ -2120,31 +2097,31 @@
     </row>
     <row r="7" ht="48" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A7" s="2" t="s">
+        <v>68</v>
+      </c>
+      <c r="B7" s="2" t="s">
+        <v>69</v>
+      </c>
+      <c r="C7" s="2" t="s">
         <v>70</v>
       </c>
-      <c r="B7" s="2" t="s">
+      <c r="D7" s="2" t="s">
+        <v>46</v>
+      </c>
+      <c r="E7" s="2" t="s">
         <v>71</v>
       </c>
-      <c r="C7" s="2" t="s">
+      <c r="F7" s="2" t="s">
         <v>72</v>
       </c>
-      <c r="D7" s="2" t="s">
-        <v>48</v>
-      </c>
-      <c r="E7" s="2" t="s">
-        <v>73</v>
-      </c>
-      <c r="F7" s="2" t="s">
-        <v>74</v>
-      </c>
       <c r="G7" s="2" t="s">
-        <v>63</v>
+        <v>61</v>
       </c>
       <c r="H7" s="2" t="s">
-        <v>64</v>
+        <v>62</v>
       </c>
       <c r="I7" s="2" t="s">
-        <v>44</v>
+        <v>42</v>
       </c>
       <c r="J7" s="3" t="s">
         <v>13</v>
@@ -2152,31 +2129,31 @@
     </row>
     <row r="8" ht="48" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A8" s="2" t="s">
+        <v>73</v>
+      </c>
+      <c r="B8" s="2" t="s">
+        <v>74</v>
+      </c>
+      <c r="C8" s="2" t="s">
         <v>75</v>
       </c>
-      <c r="B8" s="2" t="s">
+      <c r="D8" s="2" t="s">
+        <v>46</v>
+      </c>
+      <c r="E8" s="2" t="s">
         <v>76</v>
       </c>
-      <c r="C8" s="2" t="s">
+      <c r="F8" s="2" t="s">
         <v>77</v>
       </c>
-      <c r="D8" s="2" t="s">
-        <v>48</v>
-      </c>
-      <c r="E8" s="2" t="s">
+      <c r="G8" s="2" t="s">
         <v>78</v>
       </c>
-      <c r="F8" s="2" t="s">
-        <v>79</v>
-      </c>
-      <c r="G8" s="2" t="s">
-        <v>80</v>
-      </c>
       <c r="H8" s="2" t="s">
-        <v>64</v>
+        <v>62</v>
       </c>
       <c r="I8" s="2" t="s">
-        <v>44</v>
+        <v>42</v>
       </c>
       <c r="J8" s="3" t="s">
         <v>13</v>
@@ -2184,31 +2161,31 @@
     </row>
     <row r="9" ht="48" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A9" s="2" t="s">
+        <v>79</v>
+      </c>
+      <c r="B9" s="2" t="s">
+        <v>80</v>
+      </c>
+      <c r="C9" s="2" t="s">
         <v>81</v>
       </c>
-      <c r="B9" s="2" t="s">
+      <c r="D9" s="2" t="s">
+        <v>46</v>
+      </c>
+      <c r="E9" s="2" t="s">
         <v>82</v>
       </c>
-      <c r="C9" s="2" t="s">
+      <c r="F9" s="2" t="s">
         <v>83</v>
       </c>
-      <c r="D9" s="2" t="s">
-        <v>48</v>
-      </c>
-      <c r="E9" s="2" t="s">
-        <v>84</v>
-      </c>
-      <c r="F9" s="2" t="s">
-        <v>85</v>
-      </c>
       <c r="G9" s="2" t="s">
-        <v>80</v>
+        <v>78</v>
       </c>
       <c r="H9" s="2" t="s">
-        <v>64</v>
+        <v>62</v>
       </c>
       <c r="I9" s="2" t="s">
-        <v>44</v>
+        <v>42</v>
       </c>
       <c r="J9" s="3" t="s">
         <v>13</v>
@@ -2216,31 +2193,31 @@
     </row>
     <row r="10" ht="48" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A10" s="2" t="s">
+        <v>84</v>
+      </c>
+      <c r="B10" s="2" t="s">
+        <v>85</v>
+      </c>
+      <c r="C10" s="2" t="s">
         <v>86</v>
       </c>
-      <c r="B10" s="2" t="s">
+      <c r="D10" s="2" t="s">
+        <v>46</v>
+      </c>
+      <c r="E10" s="2" t="s">
         <v>87</v>
       </c>
-      <c r="C10" s="2" t="s">
+      <c r="F10" s="2" t="s">
         <v>88</v>
       </c>
-      <c r="D10" s="2" t="s">
-        <v>48</v>
-      </c>
-      <c r="E10" s="2" t="s">
+      <c r="G10" s="2" t="s">
         <v>89</v>
       </c>
-      <c r="F10" s="2" t="s">
-        <v>90</v>
-      </c>
-      <c r="G10" s="2" t="s">
-        <v>91</v>
-      </c>
       <c r="H10" s="2" t="s">
-        <v>90</v>
+        <v>88</v>
       </c>
       <c r="I10" s="2" t="s">
-        <v>44</v>
+        <v>42</v>
       </c>
       <c r="J10" s="3" t="s">
         <v>13</v>
@@ -2248,31 +2225,31 @@
     </row>
     <row r="11" ht="48" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A11" s="2" t="s">
+        <v>90</v>
+      </c>
+      <c r="B11" s="2" t="s">
+        <v>85</v>
+      </c>
+      <c r="C11" s="2" t="s">
+        <v>91</v>
+      </c>
+      <c r="D11" s="2" t="s">
         <v>92</v>
       </c>
-      <c r="B11" s="2" t="s">
-        <v>87</v>
-      </c>
-      <c r="C11" s="2" t="s">
+      <c r="E11" s="2" t="s">
         <v>93</v>
       </c>
-      <c r="D11" s="2" t="s">
+      <c r="F11" s="2" t="s">
         <v>94</v>
       </c>
-      <c r="E11" s="2" t="s">
+      <c r="G11" s="2" t="s">
         <v>95</v>
       </c>
-      <c r="F11" s="2" t="s">
-        <v>96</v>
-      </c>
-      <c r="G11" s="2" t="s">
-        <v>97</v>
-      </c>
       <c r="H11" s="2" t="s">
-        <v>90</v>
+        <v>88</v>
       </c>
       <c r="I11" s="2" t="s">
-        <v>44</v>
+        <v>42</v>
       </c>
       <c r="J11" s="3" t="s">
         <v>13</v>
@@ -2280,31 +2257,31 @@
     </row>
     <row r="12" ht="48" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A12" s="2" t="s">
+        <v>96</v>
+      </c>
+      <c r="B12" s="2" t="s">
+        <v>85</v>
+      </c>
+      <c r="C12" s="2" t="s">
+        <v>97</v>
+      </c>
+      <c r="D12" s="2" t="s">
         <v>98</v>
       </c>
-      <c r="B12" s="2" t="s">
-        <v>87</v>
-      </c>
-      <c r="C12" s="2" t="s">
+      <c r="E12" s="2" t="s">
         <v>99</v>
       </c>
-      <c r="D12" s="2" t="s">
+      <c r="F12" s="2" t="s">
+        <v>39</v>
+      </c>
+      <c r="G12" s="2" t="s">
         <v>100</v>
       </c>
-      <c r="E12" s="2" t="s">
+      <c r="H12" s="2" t="s">
         <v>101</v>
       </c>
-      <c r="F12" s="2" t="s">
-        <v>41</v>
-      </c>
-      <c r="G12" s="2" t="s">
-        <v>102</v>
-      </c>
-      <c r="H12" s="2" t="s">
-        <v>103</v>
-      </c>
       <c r="I12" s="2" t="s">
-        <v>44</v>
+        <v>42</v>
       </c>
       <c r="J12" s="3" t="s">
         <v>13</v>
@@ -2312,63 +2289,63 @@
     </row>
     <row r="13" ht="48" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A13" s="2" t="s">
+        <v>102</v>
+      </c>
+      <c r="B13" s="2" t="s">
+        <v>103</v>
+      </c>
+      <c r="C13" s="2" t="s">
         <v>104</v>
       </c>
-      <c r="B13" s="2" t="s">
+      <c r="D13" s="2" t="s">
+        <v>46</v>
+      </c>
+      <c r="E13" s="2" t="s">
         <v>105</v>
       </c>
-      <c r="C13" s="2" t="s">
+      <c r="F13" s="2" t="s">
+        <v>88</v>
+      </c>
+      <c r="G13" s="2" t="s">
         <v>106</v>
       </c>
-      <c r="D13" s="2" t="s">
-        <v>48</v>
-      </c>
-      <c r="E13" s="2" t="s">
+      <c r="H13" s="2" t="s">
+        <v>88</v>
+      </c>
+      <c r="I13" s="2" t="s">
         <v>107</v>
       </c>
-      <c r="F13" s="2" t="s">
-        <v>90</v>
-      </c>
-      <c r="G13" s="2" t="s">
-        <v>108</v>
-      </c>
-      <c r="H13" s="2" t="s">
-        <v>90</v>
-      </c>
-      <c r="I13" s="2" t="s">
-        <v>109</v>
-      </c>
-      <c r="J13" s="6" t="s">
+      <c r="J13" s="5" t="s">
         <v>4</v>
       </c>
     </row>
     <row r="14" ht="48" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A14" s="2" t="s">
+        <v>108</v>
+      </c>
+      <c r="B14" s="2" t="s">
+        <v>109</v>
+      </c>
+      <c r="C14" s="2" t="s">
         <v>110</v>
       </c>
-      <c r="B14" s="2" t="s">
+      <c r="D14" s="2" t="s">
+        <v>46</v>
+      </c>
+      <c r="E14" s="2" t="s">
         <v>111</v>
       </c>
-      <c r="C14" s="2" t="s">
+      <c r="F14" s="2" t="s">
+        <v>88</v>
+      </c>
+      <c r="G14" s="2" t="s">
         <v>112</v>
       </c>
-      <c r="D14" s="2" t="s">
-        <v>48</v>
-      </c>
-      <c r="E14" s="2" t="s">
+      <c r="H14" s="2" t="s">
         <v>113</v>
       </c>
-      <c r="F14" s="2" t="s">
-        <v>90</v>
-      </c>
-      <c r="G14" s="2" t="s">
-        <v>114</v>
-      </c>
-      <c r="H14" s="2" t="s">
-        <v>115</v>
-      </c>
       <c r="I14" s="2" t="s">
-        <v>44</v>
+        <v>42</v>
       </c>
       <c r="J14" s="3" t="s">
         <v>13</v>
@@ -2376,31 +2353,31 @@
     </row>
     <row r="15" ht="48" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A15" s="2" t="s">
+        <v>114</v>
+      </c>
+      <c r="B15" s="2" t="s">
+        <v>109</v>
+      </c>
+      <c r="C15" s="2" t="s">
+        <v>115</v>
+      </c>
+      <c r="D15" s="2" t="s">
+        <v>46</v>
+      </c>
+      <c r="E15" s="2" t="s">
         <v>116</v>
       </c>
-      <c r="B15" s="2" t="s">
-        <v>111</v>
-      </c>
-      <c r="C15" s="2" t="s">
+      <c r="F15" s="2" t="s">
+        <v>88</v>
+      </c>
+      <c r="G15" s="2" t="s">
         <v>117</v>
       </c>
-      <c r="D15" s="2" t="s">
-        <v>48</v>
-      </c>
-      <c r="E15" s="2" t="s">
+      <c r="H15" s="2" t="s">
         <v>118</v>
       </c>
-      <c r="F15" s="2" t="s">
-        <v>90</v>
-      </c>
-      <c r="G15" s="2" t="s">
-        <v>119</v>
-      </c>
-      <c r="H15" s="2" t="s">
-        <v>120</v>
-      </c>
       <c r="I15" s="2" t="s">
-        <v>44</v>
+        <v>42</v>
       </c>
       <c r="J15" s="3" t="s">
         <v>13</v>
@@ -2408,31 +2385,31 @@
     </row>
     <row r="16" ht="48" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A16" s="2" t="s">
+        <v>119</v>
+      </c>
+      <c r="B16" s="2" t="s">
+        <v>109</v>
+      </c>
+      <c r="C16" s="2" t="s">
+        <v>120</v>
+      </c>
+      <c r="D16" s="2" t="s">
+        <v>46</v>
+      </c>
+      <c r="E16" s="2" t="s">
         <v>121</v>
       </c>
-      <c r="B16" s="2" t="s">
-        <v>111</v>
-      </c>
-      <c r="C16" s="2" t="s">
+      <c r="F16" s="2" t="s">
+        <v>88</v>
+      </c>
+      <c r="G16" s="2" t="s">
         <v>122</v>
       </c>
-      <c r="D16" s="2" t="s">
-        <v>48</v>
-      </c>
-      <c r="E16" s="2" t="s">
+      <c r="H16" s="2" t="s">
         <v>123</v>
       </c>
-      <c r="F16" s="2" t="s">
-        <v>90</v>
-      </c>
-      <c r="G16" s="2" t="s">
-        <v>124</v>
-      </c>
-      <c r="H16" s="2" t="s">
-        <v>125</v>
-      </c>
       <c r="I16" s="2" t="s">
-        <v>44</v>
+        <v>42</v>
       </c>
       <c r="J16" s="3" t="s">
         <v>13</v>
@@ -2440,127 +2417,127 @@
     </row>
     <row r="17" ht="48" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A17" s="2" t="s">
+        <v>124</v>
+      </c>
+      <c r="B17" s="2" t="s">
+        <v>125</v>
+      </c>
+      <c r="C17" s="2" t="s">
         <v>126</v>
       </c>
-      <c r="B17" s="2" t="s">
+      <c r="D17" s="2" t="s">
+        <v>46</v>
+      </c>
+      <c r="E17" s="2" t="s">
         <v>127</v>
       </c>
-      <c r="C17" s="2" t="s">
+      <c r="F17" s="2" t="s">
         <v>128</v>
       </c>
-      <c r="D17" s="2" t="s">
-        <v>48</v>
-      </c>
-      <c r="E17" s="2" t="s">
+      <c r="G17" s="2" t="s">
         <v>129</v>
       </c>
-      <c r="F17" s="2" t="s">
-        <v>130</v>
-      </c>
-      <c r="G17" s="2" t="s">
-        <v>131</v>
-      </c>
       <c r="H17" s="2" t="s">
-        <v>90</v>
+        <v>88</v>
       </c>
       <c r="I17" s="2" t="s">
-        <v>109</v>
-      </c>
-      <c r="J17" s="6" t="s">
+        <v>107</v>
+      </c>
+      <c r="J17" s="5" t="s">
         <v>4</v>
       </c>
     </row>
     <row r="18" ht="48" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A18" s="2" t="s">
+        <v>130</v>
+      </c>
+      <c r="B18" s="2" t="s">
+        <v>125</v>
+      </c>
+      <c r="C18" s="2" t="s">
+        <v>131</v>
+      </c>
+      <c r="D18" s="2" t="s">
+        <v>46</v>
+      </c>
+      <c r="E18" s="2" t="s">
         <v>132</v>
       </c>
-      <c r="B18" s="2" t="s">
-        <v>127</v>
-      </c>
-      <c r="C18" s="2" t="s">
+      <c r="F18" s="2" t="s">
         <v>133</v>
       </c>
-      <c r="D18" s="2" t="s">
-        <v>48</v>
-      </c>
-      <c r="E18" s="2" t="s">
+      <c r="G18" s="2" t="s">
         <v>134</v>
       </c>
-      <c r="F18" s="2" t="s">
-        <v>135</v>
-      </c>
-      <c r="G18" s="2" t="s">
-        <v>136</v>
-      </c>
       <c r="H18" s="2" t="s">
-        <v>103</v>
+        <v>101</v>
       </c>
       <c r="I18" s="2" t="s">
-        <v>109</v>
-      </c>
-      <c r="J18" s="6" t="s">
+        <v>107</v>
+      </c>
+      <c r="J18" s="5" t="s">
         <v>4</v>
       </c>
     </row>
     <row r="19" ht="48" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A19" s="2" t="s">
+        <v>135</v>
+      </c>
+      <c r="B19" s="2" t="s">
+        <v>125</v>
+      </c>
+      <c r="C19" s="2" t="s">
+        <v>136</v>
+      </c>
+      <c r="D19" s="2" t="s">
+        <v>46</v>
+      </c>
+      <c r="E19" s="2" t="s">
         <v>137</v>
       </c>
-      <c r="B19" s="2" t="s">
-        <v>127</v>
-      </c>
-      <c r="C19" s="2" t="s">
+      <c r="F19" s="2" t="s">
         <v>138</v>
       </c>
-      <c r="D19" s="2" t="s">
-        <v>48</v>
-      </c>
-      <c r="E19" s="2" t="s">
+      <c r="G19" s="2" t="s">
         <v>139</v>
       </c>
-      <c r="F19" s="2" t="s">
-        <v>140</v>
-      </c>
-      <c r="G19" s="2" t="s">
-        <v>141</v>
-      </c>
       <c r="H19" s="2" t="s">
-        <v>64</v>
+        <v>62</v>
       </c>
       <c r="I19" s="2" t="s">
-        <v>109</v>
-      </c>
-      <c r="J19" s="6" t="s">
+        <v>107</v>
+      </c>
+      <c r="J19" s="5" t="s">
         <v>4</v>
       </c>
     </row>
     <row r="20" ht="48" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A20" s="2" t="s">
+        <v>140</v>
+      </c>
+      <c r="B20" s="2" t="s">
+        <v>141</v>
+      </c>
+      <c r="C20" s="2" t="s">
         <v>142</v>
       </c>
-      <c r="B20" s="2" t="s">
+      <c r="D20" s="2" t="s">
+        <v>46</v>
+      </c>
+      <c r="E20" s="2" t="s">
         <v>143</v>
       </c>
-      <c r="C20" s="2" t="s">
+      <c r="F20" s="2" t="s">
+        <v>88</v>
+      </c>
+      <c r="G20" s="2" t="s">
         <v>144</v>
       </c>
-      <c r="D20" s="2" t="s">
-        <v>48</v>
-      </c>
-      <c r="E20" s="2" t="s">
-        <v>145</v>
-      </c>
-      <c r="F20" s="2" t="s">
-        <v>90</v>
-      </c>
-      <c r="G20" s="2" t="s">
-        <v>146</v>
-      </c>
       <c r="H20" s="2" t="s">
-        <v>90</v>
+        <v>88</v>
       </c>
       <c r="I20" s="2" t="s">
-        <v>44</v>
+        <v>42</v>
       </c>
       <c r="J20" s="3" t="s">
         <v>13</v>
@@ -2568,97 +2545,97 @@
     </row>
     <row r="21" ht="48" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A21" s="2" t="s">
+        <v>145</v>
+      </c>
+      <c r="B21" s="2" t="s">
+        <v>141</v>
+      </c>
+      <c r="C21" s="2" t="s">
+        <v>146</v>
+      </c>
+      <c r="D21" s="2" t="s">
+        <v>46</v>
+      </c>
+      <c r="E21" s="2" t="s">
         <v>147</v>
       </c>
-      <c r="B21" s="2" t="s">
-        <v>143</v>
-      </c>
-      <c r="C21" s="2" t="s">
+      <c r="F21" s="2" t="s">
+        <v>39</v>
+      </c>
+      <c r="G21" s="2" t="s">
         <v>148</v>
       </c>
-      <c r="D21" s="2" t="s">
-        <v>48</v>
-      </c>
-      <c r="E21" s="2" t="s">
+      <c r="H21" s="2" t="s">
         <v>149</v>
       </c>
-      <c r="F21" s="2" t="s">
-        <v>41</v>
-      </c>
-      <c r="G21" s="2" t="s">
-        <v>150</v>
-      </c>
-      <c r="H21" s="2" t="s">
-        <v>151</v>
-      </c>
       <c r="I21" s="2" t="s">
-        <v>109</v>
-      </c>
-      <c r="J21" s="6" t="s">
+        <v>107</v>
+      </c>
+      <c r="J21" s="5" t="s">
         <v>4</v>
       </c>
     </row>
     <row r="22" ht="48" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A22" s="2" t="s">
+        <v>150</v>
+      </c>
+      <c r="B22" s="2" t="s">
+        <v>141</v>
+      </c>
+      <c r="C22" s="2" t="s">
+        <v>151</v>
+      </c>
+      <c r="D22" s="2" t="s">
+        <v>46</v>
+      </c>
+      <c r="E22" s="2" t="s">
         <v>152</v>
       </c>
-      <c r="B22" s="2" t="s">
-        <v>143</v>
-      </c>
-      <c r="C22" s="2" t="s">
+      <c r="F22" s="2" t="s">
         <v>153</v>
       </c>
-      <c r="D22" s="2" t="s">
-        <v>48</v>
-      </c>
-      <c r="E22" s="2" t="s">
+      <c r="G22" s="2" t="s">
         <v>154</v>
       </c>
-      <c r="F22" s="2" t="s">
-        <v>155</v>
-      </c>
-      <c r="G22" s="2" t="s">
-        <v>156</v>
-      </c>
       <c r="H22" s="2" t="s">
-        <v>64</v>
+        <v>62</v>
       </c>
       <c r="I22" s="2" t="s">
-        <v>109</v>
-      </c>
-      <c r="J22" s="6" t="s">
+        <v>107</v>
+      </c>
+      <c r="J22" s="5" t="s">
         <v>4</v>
       </c>
     </row>
     <row r="23" ht="48" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A23" s="2" t="s">
+        <v>155</v>
+      </c>
+      <c r="B23" s="2" t="s">
+        <v>141</v>
+      </c>
+      <c r="C23" s="2" t="s">
+        <v>156</v>
+      </c>
+      <c r="D23" s="2" t="s">
+        <v>46</v>
+      </c>
+      <c r="E23" s="2" t="s">
         <v>157</v>
       </c>
-      <c r="B23" s="2" t="s">
-        <v>143</v>
-      </c>
-      <c r="C23" s="2" t="s">
+      <c r="F23" s="2" t="s">
         <v>158</v>
       </c>
-      <c r="D23" s="2" t="s">
-        <v>48</v>
-      </c>
-      <c r="E23" s="2" t="s">
+      <c r="G23" s="2" t="s">
         <v>159</v>
       </c>
-      <c r="F23" s="2" t="s">
+      <c r="H23" s="2" t="s">
         <v>160</v>
       </c>
-      <c r="G23" s="2" t="s">
-        <v>161</v>
-      </c>
-      <c r="H23" s="2" t="s">
-        <v>162</v>
-      </c>
       <c r="I23" s="2" t="s">
-        <v>109</v>
-      </c>
-      <c r="J23" s="6" t="s">
+        <v>107</v>
+      </c>
+      <c r="J23" s="5" t="s">
         <v>4</v>
       </c>
     </row>
@@ -2687,66 +2664,66 @@
   <sheetData>
     <row r="1" ht="28" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
+        <v>24</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>25</v>
+      </c>
+      <c r="C1" s="1" t="s">
         <v>26</v>
       </c>
-      <c r="B1" s="1" t="s">
+      <c r="D1" s="1" t="s">
         <v>27</v>
       </c>
-      <c r="C1" s="1" t="s">
+      <c r="E1" s="1" t="s">
         <v>28</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="F1" s="1" t="s">
         <v>29</v>
       </c>
-      <c r="E1" s="1" t="s">
+      <c r="G1" s="1" t="s">
         <v>30</v>
       </c>
-      <c r="F1" s="1" t="s">
+      <c r="H1" s="1" t="s">
         <v>31</v>
       </c>
-      <c r="G1" s="1" t="s">
+      <c r="I1" s="1" t="s">
         <v>32</v>
       </c>
-      <c r="H1" s="1" t="s">
+      <c r="J1" s="1" t="s">
         <v>33</v>
-      </c>
-      <c r="I1" s="1" t="s">
-        <v>34</v>
-      </c>
-      <c r="J1" s="1" t="s">
-        <v>35</v>
       </c>
     </row>
     <row r="2" ht="240" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A2" s="2" t="s">
+        <v>161</v>
+      </c>
+      <c r="B2" s="2" t="s">
+        <v>162</v>
+      </c>
+      <c r="C2" s="2" t="s">
         <v>163</v>
       </c>
-      <c r="B2" s="2" t="s">
+      <c r="D2" s="2" t="s">
         <v>164</v>
       </c>
-      <c r="C2" s="2" t="s">
+      <c r="E2" s="2" t="s">
         <v>165</v>
       </c>
-      <c r="D2" s="2" t="s">
+      <c r="F2" s="2" t="s">
         <v>166</v>
       </c>
-      <c r="E2" s="2" t="s">
+      <c r="G2" s="2" t="s">
         <v>167</v>
       </c>
-      <c r="F2" s="2" t="s">
+      <c r="H2" s="2" t="s">
         <v>168</v>
       </c>
-      <c r="G2" s="2" t="s">
-        <v>169</v>
-      </c>
-      <c r="H2" s="2" t="s">
-        <v>170</v>
-      </c>
       <c r="I2" s="2" t="s">
-        <v>171</v>
-      </c>
-      <c r="J2" s="4" t="s">
-        <v>17</v>
+        <v>42</v>
+      </c>
+      <c r="J2" s="3" t="s">
+        <v>13</v>
       </c>
     </row>
   </sheetData>
@@ -2774,63 +2751,63 @@
   <sheetData>
     <row r="1" ht="28" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
+        <v>24</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>25</v>
+      </c>
+      <c r="C1" s="1" t="s">
         <v>26</v>
       </c>
-      <c r="B1" s="1" t="s">
+      <c r="D1" s="1" t="s">
         <v>27</v>
       </c>
-      <c r="C1" s="1" t="s">
+      <c r="E1" s="1" t="s">
         <v>28</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="F1" s="1" t="s">
         <v>29</v>
       </c>
-      <c r="E1" s="1" t="s">
+      <c r="G1" s="1" t="s">
         <v>30</v>
       </c>
-      <c r="F1" s="1" t="s">
+      <c r="H1" s="1" t="s">
         <v>31</v>
       </c>
-      <c r="G1" s="1" t="s">
+      <c r="I1" s="1" t="s">
         <v>32</v>
       </c>
-      <c r="H1" s="1" t="s">
+      <c r="J1" s="1" t="s">
         <v>33</v>
-      </c>
-      <c r="I1" s="1" t="s">
-        <v>34</v>
-      </c>
-      <c r="J1" s="1" t="s">
-        <v>35</v>
       </c>
     </row>
     <row r="2" ht="64" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A2" s="2" t="s">
+        <v>169</v>
+      </c>
+      <c r="B2" s="2" t="s">
+        <v>170</v>
+      </c>
+      <c r="C2" s="2" t="s">
+        <v>171</v>
+      </c>
+      <c r="D2" s="2" t="s">
         <v>172</v>
       </c>
-      <c r="B2" s="2" t="s">
+      <c r="E2" s="2" t="s">
         <v>173</v>
       </c>
-      <c r="C2" s="2" t="s">
+      <c r="F2" s="2" t="s">
         <v>174</v>
       </c>
-      <c r="D2" s="2" t="s">
+      <c r="G2" s="2" t="s">
         <v>175</v>
       </c>
-      <c r="E2" s="2" t="s">
+      <c r="H2" s="2" t="s">
         <v>176</v>
       </c>
-      <c r="F2" s="2" t="s">
-        <v>177</v>
-      </c>
-      <c r="G2" s="2" t="s">
-        <v>178</v>
-      </c>
-      <c r="H2" s="2" t="s">
-        <v>179</v>
-      </c>
       <c r="I2" s="2" t="s">
-        <v>44</v>
+        <v>42</v>
       </c>
       <c r="J2" s="3" t="s">
         <v>13</v>
@@ -2838,31 +2815,31 @@
     </row>
     <row r="3" ht="64" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A3" s="2" t="s">
+        <v>177</v>
+      </c>
+      <c r="B3" s="2" t="s">
+        <v>178</v>
+      </c>
+      <c r="C3" s="2" t="s">
+        <v>179</v>
+      </c>
+      <c r="D3" s="2" t="s">
         <v>180</v>
       </c>
-      <c r="B3" s="2" t="s">
+      <c r="E3" s="2" t="s">
         <v>181</v>
       </c>
-      <c r="C3" s="2" t="s">
+      <c r="F3" s="2" t="s">
         <v>182</v>
       </c>
-      <c r="D3" s="2" t="s">
+      <c r="G3" s="2" t="s">
         <v>183</v>
       </c>
-      <c r="E3" s="2" t="s">
+      <c r="H3" s="2" t="s">
         <v>184</v>
       </c>
-      <c r="F3" s="2" t="s">
-        <v>185</v>
-      </c>
-      <c r="G3" s="2" t="s">
-        <v>186</v>
-      </c>
-      <c r="H3" s="2" t="s">
-        <v>187</v>
-      </c>
       <c r="I3" s="2" t="s">
-        <v>44</v>
+        <v>42</v>
       </c>
       <c r="J3" s="3" t="s">
         <v>13</v>
@@ -2870,31 +2847,31 @@
     </row>
     <row r="4" ht="48" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A4" s="2" t="s">
+        <v>185</v>
+      </c>
+      <c r="B4" s="2" t="s">
+        <v>186</v>
+      </c>
+      <c r="C4" s="2" t="s">
+        <v>187</v>
+      </c>
+      <c r="D4" s="2" t="s">
         <v>188</v>
       </c>
-      <c r="B4" s="2" t="s">
+      <c r="E4" s="2" t="s">
         <v>189</v>
       </c>
-      <c r="C4" s="2" t="s">
+      <c r="F4" s="2" t="s">
         <v>190</v>
       </c>
-      <c r="D4" s="2" t="s">
+      <c r="G4" s="2" t="s">
         <v>191</v>
       </c>
-      <c r="E4" s="2" t="s">
+      <c r="H4" s="2" t="s">
         <v>192</v>
       </c>
-      <c r="F4" s="2" t="s">
-        <v>193</v>
-      </c>
-      <c r="G4" s="2" t="s">
-        <v>194</v>
-      </c>
-      <c r="H4" s="2" t="s">
-        <v>195</v>
-      </c>
       <c r="I4" s="2" t="s">
-        <v>44</v>
+        <v>42</v>
       </c>
       <c r="J4" s="3" t="s">
         <v>13</v>
@@ -2902,63 +2879,63 @@
     </row>
     <row r="5" ht="48" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A5" s="2" t="s">
+        <v>193</v>
+      </c>
+      <c r="B5" s="2" t="s">
+        <v>194</v>
+      </c>
+      <c r="C5" s="2" t="s">
+        <v>195</v>
+      </c>
+      <c r="D5" s="2" t="s">
+        <v>188</v>
+      </c>
+      <c r="E5" s="2" t="s">
         <v>196</v>
       </c>
-      <c r="B5" s="2" t="s">
+      <c r="F5" s="2" t="s">
         <v>197</v>
       </c>
-      <c r="C5" s="2" t="s">
-        <v>198</v>
-      </c>
-      <c r="D5" s="2" t="s">
+      <c r="G5" s="2" t="s">
         <v>191</v>
       </c>
-      <c r="E5" s="2" t="s">
-        <v>199</v>
-      </c>
-      <c r="F5" s="2" t="s">
-        <v>200</v>
-      </c>
-      <c r="G5" s="2" t="s">
-        <v>194</v>
-      </c>
       <c r="H5" s="2" t="s">
-        <v>195</v>
+        <v>192</v>
       </c>
       <c r="I5" s="2" t="s">
-        <v>109</v>
-      </c>
-      <c r="J5" s="6" t="s">
+        <v>107</v>
+      </c>
+      <c r="J5" s="5" t="s">
         <v>4</v>
       </c>
     </row>
     <row r="6" ht="48" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A6" s="2" t="s">
+        <v>198</v>
+      </c>
+      <c r="B6" s="2" t="s">
+        <v>199</v>
+      </c>
+      <c r="C6" s="2" t="s">
+        <v>200</v>
+      </c>
+      <c r="D6" s="2" t="s">
+        <v>188</v>
+      </c>
+      <c r="E6" s="2" t="s">
         <v>201</v>
       </c>
-      <c r="B6" s="2" t="s">
+      <c r="F6" s="2" t="s">
         <v>202</v>
       </c>
-      <c r="C6" s="2" t="s">
-        <v>203</v>
-      </c>
-      <c r="D6" s="2" t="s">
+      <c r="G6" s="2" t="s">
         <v>191</v>
       </c>
-      <c r="E6" s="2" t="s">
-        <v>204</v>
-      </c>
-      <c r="F6" s="2" t="s">
-        <v>205</v>
-      </c>
-      <c r="G6" s="2" t="s">
-        <v>194</v>
-      </c>
       <c r="H6" s="2" t="s">
-        <v>195</v>
+        <v>192</v>
       </c>
       <c r="I6" s="2" t="s">
-        <v>44</v>
+        <v>42</v>
       </c>
       <c r="J6" s="3" t="s">
         <v>13</v>
@@ -2966,31 +2943,31 @@
     </row>
     <row r="7" ht="48" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A7" s="2" t="s">
+        <v>203</v>
+      </c>
+      <c r="B7" s="2" t="s">
+        <v>204</v>
+      </c>
+      <c r="C7" s="2" t="s">
+        <v>205</v>
+      </c>
+      <c r="D7" s="2" t="s">
+        <v>188</v>
+      </c>
+      <c r="E7" s="2" t="s">
         <v>206</v>
       </c>
-      <c r="B7" s="2" t="s">
+      <c r="F7" s="2" t="s">
         <v>207</v>
       </c>
-      <c r="C7" s="2" t="s">
+      <c r="G7" s="2" t="s">
         <v>208</v>
       </c>
-      <c r="D7" s="2" t="s">
-        <v>191</v>
-      </c>
-      <c r="E7" s="2" t="s">
-        <v>209</v>
-      </c>
-      <c r="F7" s="2" t="s">
-        <v>210</v>
-      </c>
-      <c r="G7" s="2" t="s">
-        <v>211</v>
-      </c>
       <c r="H7" s="2" t="s">
-        <v>195</v>
+        <v>192</v>
       </c>
       <c r="I7" s="2" t="s">
-        <v>44</v>
+        <v>42</v>
       </c>
       <c r="J7" s="3" t="s">
         <v>13</v>
@@ -2998,95 +2975,95 @@
     </row>
     <row r="8" ht="48" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A8" s="2" t="s">
+        <v>209</v>
+      </c>
+      <c r="B8" s="2" t="s">
+        <v>210</v>
+      </c>
+      <c r="C8" s="2" t="s">
+        <v>211</v>
+      </c>
+      <c r="D8" s="2" t="s">
+        <v>188</v>
+      </c>
+      <c r="E8" s="2" t="s">
         <v>212</v>
       </c>
-      <c r="B8" s="2" t="s">
+      <c r="F8" s="2" t="s">
         <v>213</v>
       </c>
-      <c r="C8" s="2" t="s">
+      <c r="G8" s="2" t="s">
         <v>214</v>
       </c>
-      <c r="D8" s="2" t="s">
-        <v>191</v>
-      </c>
-      <c r="E8" s="2" t="s">
-        <v>215</v>
-      </c>
-      <c r="F8" s="2" t="s">
-        <v>216</v>
-      </c>
-      <c r="G8" s="2" t="s">
-        <v>217</v>
-      </c>
       <c r="H8" s="2" t="s">
-        <v>195</v>
+        <v>192</v>
       </c>
       <c r="I8" s="2" t="s">
-        <v>109</v>
-      </c>
-      <c r="J8" s="6" t="s">
+        <v>107</v>
+      </c>
+      <c r="J8" s="5" t="s">
         <v>4</v>
       </c>
     </row>
     <row r="9" ht="48" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A9" s="2" t="s">
+        <v>215</v>
+      </c>
+      <c r="B9" s="2" t="s">
+        <v>216</v>
+      </c>
+      <c r="C9" s="2" t="s">
+        <v>217</v>
+      </c>
+      <c r="D9" s="2" t="s">
         <v>218</v>
       </c>
-      <c r="B9" s="2" t="s">
+      <c r="E9" s="2" t="s">
         <v>219</v>
       </c>
-      <c r="C9" s="2" t="s">
+      <c r="F9" s="2" t="s">
         <v>220</v>
       </c>
-      <c r="D9" s="2" t="s">
+      <c r="G9" s="2" t="s">
         <v>221</v>
       </c>
-      <c r="E9" s="2" t="s">
+      <c r="H9" s="2" t="s">
         <v>222</v>
       </c>
-      <c r="F9" s="2" t="s">
-        <v>223</v>
-      </c>
-      <c r="G9" s="2" t="s">
-        <v>224</v>
-      </c>
-      <c r="H9" s="2" t="s">
-        <v>225</v>
-      </c>
       <c r="I9" s="2" t="s">
-        <v>109</v>
-      </c>
-      <c r="J9" s="6" t="s">
+        <v>107</v>
+      </c>
+      <c r="J9" s="5" t="s">
         <v>4</v>
       </c>
     </row>
     <row r="10" ht="48" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A10" s="2" t="s">
+        <v>223</v>
+      </c>
+      <c r="B10" s="2" t="s">
+        <v>224</v>
+      </c>
+      <c r="C10" s="2" t="s">
+        <v>225</v>
+      </c>
+      <c r="D10" s="2" t="s">
+        <v>188</v>
+      </c>
+      <c r="E10" s="2" t="s">
         <v>226</v>
       </c>
-      <c r="B10" s="2" t="s">
+      <c r="F10" s="2" t="s">
         <v>227</v>
       </c>
-      <c r="C10" s="2" t="s">
+      <c r="G10" s="2" t="s">
         <v>228</v>
       </c>
-      <c r="D10" s="2" t="s">
-        <v>191</v>
-      </c>
-      <c r="E10" s="2" t="s">
-        <v>229</v>
-      </c>
-      <c r="F10" s="2" t="s">
-        <v>230</v>
-      </c>
-      <c r="G10" s="2" t="s">
-        <v>231</v>
-      </c>
       <c r="H10" s="2" t="s">
-        <v>90</v>
+        <v>88</v>
       </c>
       <c r="I10" s="2" t="s">
-        <v>44</v>
+        <v>42</v>
       </c>
       <c r="J10" s="3" t="s">
         <v>13</v>
@@ -3094,31 +3071,31 @@
     </row>
     <row r="11" ht="64" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A11" s="2" t="s">
+        <v>229</v>
+      </c>
+      <c r="B11" s="2" t="s">
+        <v>230</v>
+      </c>
+      <c r="C11" s="2" t="s">
+        <v>231</v>
+      </c>
+      <c r="D11" s="2" t="s">
         <v>232</v>
       </c>
-      <c r="B11" s="2" t="s">
+      <c r="E11" s="2" t="s">
         <v>233</v>
       </c>
-      <c r="C11" s="2" t="s">
+      <c r="F11" s="2" t="s">
         <v>234</v>
       </c>
-      <c r="D11" s="2" t="s">
+      <c r="G11" s="2" t="s">
         <v>235</v>
       </c>
-      <c r="E11" s="2" t="s">
+      <c r="H11" s="2" t="s">
         <v>236</v>
       </c>
-      <c r="F11" s="2" t="s">
-        <v>237</v>
-      </c>
-      <c r="G11" s="2" t="s">
-        <v>238</v>
-      </c>
-      <c r="H11" s="2" t="s">
-        <v>239</v>
-      </c>
       <c r="I11" s="2" t="s">
-        <v>44</v>
+        <v>42</v>
       </c>
       <c r="J11" s="3" t="s">
         <v>13</v>
@@ -3126,63 +3103,63 @@
     </row>
     <row r="12" ht="48" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A12" s="2" t="s">
+        <v>237</v>
+      </c>
+      <c r="B12" s="2" t="s">
+        <v>238</v>
+      </c>
+      <c r="C12" s="2" t="s">
+        <v>239</v>
+      </c>
+      <c r="D12" s="2" t="s">
+        <v>232</v>
+      </c>
+      <c r="E12" s="2" t="s">
         <v>240</v>
       </c>
-      <c r="B12" s="2" t="s">
+      <c r="F12" s="2" t="s">
         <v>241</v>
       </c>
-      <c r="C12" s="2" t="s">
+      <c r="G12" s="2" t="s">
         <v>242</v>
       </c>
-      <c r="D12" s="2" t="s">
-        <v>235</v>
-      </c>
-      <c r="E12" s="2" t="s">
-        <v>243</v>
-      </c>
-      <c r="F12" s="2" t="s">
-        <v>244</v>
-      </c>
-      <c r="G12" s="2" t="s">
-        <v>245</v>
-      </c>
       <c r="H12" s="2" t="s">
-        <v>239</v>
+        <v>236</v>
       </c>
       <c r="I12" s="2" t="s">
-        <v>109</v>
-      </c>
-      <c r="J12" s="6" t="s">
+        <v>107</v>
+      </c>
+      <c r="J12" s="5" t="s">
         <v>4</v>
       </c>
     </row>
     <row r="13" ht="48" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A13" s="2" t="s">
+        <v>243</v>
+      </c>
+      <c r="B13" s="2" t="s">
+        <v>244</v>
+      </c>
+      <c r="C13" s="2" t="s">
+        <v>245</v>
+      </c>
+      <c r="D13" s="2" t="s">
         <v>246</v>
       </c>
-      <c r="B13" s="2" t="s">
+      <c r="E13" s="2" t="s">
         <v>247</v>
       </c>
-      <c r="C13" s="2" t="s">
+      <c r="F13" s="2" t="s">
         <v>248</v>
       </c>
-      <c r="D13" s="2" t="s">
+      <c r="G13" s="2" t="s">
         <v>249</v>
       </c>
-      <c r="E13" s="2" t="s">
-        <v>250</v>
-      </c>
-      <c r="F13" s="2" t="s">
-        <v>251</v>
-      </c>
-      <c r="G13" s="2" t="s">
-        <v>252</v>
-      </c>
       <c r="H13" s="2" t="s">
-        <v>239</v>
+        <v>236</v>
       </c>
       <c r="I13" s="2" t="s">
-        <v>44</v>
+        <v>42</v>
       </c>
       <c r="J13" s="3" t="s">
         <v>13</v>
@@ -3190,31 +3167,31 @@
     </row>
     <row r="14" ht="48" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A14" s="2" t="s">
+        <v>250</v>
+      </c>
+      <c r="B14" s="2" t="s">
+        <v>251</v>
+      </c>
+      <c r="C14" s="2" t="s">
+        <v>252</v>
+      </c>
+      <c r="D14" s="2" t="s">
+        <v>188</v>
+      </c>
+      <c r="E14" s="2" t="s">
         <v>253</v>
       </c>
-      <c r="B14" s="2" t="s">
+      <c r="F14" s="2" t="s">
+        <v>88</v>
+      </c>
+      <c r="G14" s="2" t="s">
         <v>254</v>
       </c>
-      <c r="C14" s="2" t="s">
-        <v>255</v>
-      </c>
-      <c r="D14" s="2" t="s">
-        <v>191</v>
-      </c>
-      <c r="E14" s="2" t="s">
-        <v>256</v>
-      </c>
-      <c r="F14" s="2" t="s">
-        <v>90</v>
-      </c>
-      <c r="G14" s="2" t="s">
-        <v>257</v>
-      </c>
       <c r="H14" s="2" t="s">
-        <v>90</v>
+        <v>88</v>
       </c>
       <c r="I14" s="2" t="s">
-        <v>44</v>
+        <v>42</v>
       </c>
       <c r="J14" s="3" t="s">
         <v>13</v>
@@ -3222,63 +3199,63 @@
     </row>
     <row r="15" ht="48" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A15" s="2" t="s">
+        <v>255</v>
+      </c>
+      <c r="B15" s="2" t="s">
+        <v>256</v>
+      </c>
+      <c r="C15" s="2" t="s">
+        <v>257</v>
+      </c>
+      <c r="D15" s="2" t="s">
         <v>258</v>
       </c>
-      <c r="B15" s="2" t="s">
+      <c r="E15" s="2" t="s">
         <v>259</v>
       </c>
-      <c r="C15" s="2" t="s">
+      <c r="F15" s="2" t="s">
+        <v>88</v>
+      </c>
+      <c r="G15" s="2" t="s">
         <v>260</v>
       </c>
-      <c r="D15" s="2" t="s">
-        <v>261</v>
-      </c>
-      <c r="E15" s="2" t="s">
-        <v>262</v>
-      </c>
-      <c r="F15" s="2" t="s">
-        <v>90</v>
-      </c>
-      <c r="G15" s="2" t="s">
-        <v>263</v>
-      </c>
       <c r="H15" s="2" t="s">
-        <v>90</v>
+        <v>88</v>
       </c>
       <c r="I15" s="2" t="s">
-        <v>109</v>
-      </c>
-      <c r="J15" s="6" t="s">
+        <v>107</v>
+      </c>
+      <c r="J15" s="5" t="s">
         <v>4</v>
       </c>
     </row>
     <row r="16" ht="48" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A16" s="2" t="s">
+        <v>261</v>
+      </c>
+      <c r="B16" s="2" t="s">
+        <v>262</v>
+      </c>
+      <c r="C16" s="2" t="s">
+        <v>263</v>
+      </c>
+      <c r="D16" s="2" t="s">
+        <v>232</v>
+      </c>
+      <c r="E16" s="2" t="s">
         <v>264</v>
       </c>
-      <c r="B16" s="2" t="s">
-        <v>265</v>
-      </c>
-      <c r="C16" s="2" t="s">
-        <v>266</v>
-      </c>
-      <c r="D16" s="2" t="s">
-        <v>235</v>
-      </c>
-      <c r="E16" s="2" t="s">
-        <v>267</v>
-      </c>
       <c r="F16" s="2" t="s">
-        <v>96</v>
+        <v>94</v>
       </c>
       <c r="G16" s="2" t="s">
-        <v>97</v>
+        <v>95</v>
       </c>
       <c r="H16" s="2" t="s">
-        <v>90</v>
+        <v>88</v>
       </c>
       <c r="I16" s="2" t="s">
-        <v>44</v>
+        <v>42</v>
       </c>
       <c r="J16" s="3" t="s">
         <v>13</v>
@@ -3286,63 +3263,63 @@
     </row>
     <row r="17" ht="48" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A17" s="2" t="s">
+        <v>265</v>
+      </c>
+      <c r="B17" s="2" t="s">
+        <v>266</v>
+      </c>
+      <c r="C17" s="2" t="s">
+        <v>267</v>
+      </c>
+      <c r="D17" s="2" t="s">
         <v>268</v>
       </c>
-      <c r="B17" s="2" t="s">
+      <c r="E17" s="2" t="s">
         <v>269</v>
       </c>
-      <c r="C17" s="2" t="s">
+      <c r="F17" s="2" t="s">
+        <v>88</v>
+      </c>
+      <c r="G17" s="2" t="s">
         <v>270</v>
       </c>
-      <c r="D17" s="2" t="s">
+      <c r="H17" s="2" t="s">
         <v>271</v>
       </c>
-      <c r="E17" s="2" t="s">
-        <v>272</v>
-      </c>
-      <c r="F17" s="2" t="s">
-        <v>90</v>
-      </c>
-      <c r="G17" s="2" t="s">
-        <v>273</v>
-      </c>
-      <c r="H17" s="2" t="s">
-        <v>274</v>
-      </c>
       <c r="I17" s="2" t="s">
-        <v>109</v>
-      </c>
-      <c r="J17" s="6" t="s">
+        <v>107</v>
+      </c>
+      <c r="J17" s="5" t="s">
         <v>4</v>
       </c>
     </row>
     <row r="18" ht="48" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A18" s="2" t="s">
+        <v>272</v>
+      </c>
+      <c r="B18" s="2" t="s">
+        <v>273</v>
+      </c>
+      <c r="C18" s="2" t="s">
+        <v>274</v>
+      </c>
+      <c r="D18" s="2" t="s">
+        <v>188</v>
+      </c>
+      <c r="E18" s="2" t="s">
         <v>275</v>
       </c>
-      <c r="B18" s="2" t="s">
+      <c r="F18" s="2" t="s">
+        <v>88</v>
+      </c>
+      <c r="G18" s="2" t="s">
         <v>276</v>
       </c>
-      <c r="C18" s="2" t="s">
+      <c r="H18" s="2" t="s">
         <v>277</v>
       </c>
-      <c r="D18" s="2" t="s">
-        <v>191</v>
-      </c>
-      <c r="E18" s="2" t="s">
-        <v>278</v>
-      </c>
-      <c r="F18" s="2" t="s">
-        <v>90</v>
-      </c>
-      <c r="G18" s="2" t="s">
-        <v>279</v>
-      </c>
-      <c r="H18" s="2" t="s">
-        <v>280</v>
-      </c>
       <c r="I18" s="2" t="s">
-        <v>44</v>
+        <v>42</v>
       </c>
       <c r="J18" s="3" t="s">
         <v>13</v>
@@ -3350,31 +3327,31 @@
     </row>
     <row r="19" ht="48" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A19" s="2" t="s">
-        <v>281</v>
+        <v>278</v>
       </c>
       <c r="B19" s="2" t="s">
-        <v>276</v>
+        <v>273</v>
       </c>
       <c r="C19" s="2" t="s">
+        <v>120</v>
+      </c>
+      <c r="D19" s="2" t="s">
+        <v>188</v>
+      </c>
+      <c r="E19" s="2" t="s">
+        <v>121</v>
+      </c>
+      <c r="F19" s="2" t="s">
+        <v>88</v>
+      </c>
+      <c r="G19" s="2" t="s">
         <v>122</v>
       </c>
-      <c r="D19" s="2" t="s">
-        <v>191</v>
-      </c>
-      <c r="E19" s="2" t="s">
+      <c r="H19" s="2" t="s">
         <v>123</v>
       </c>
-      <c r="F19" s="2" t="s">
-        <v>90</v>
-      </c>
-      <c r="G19" s="2" t="s">
-        <v>124</v>
-      </c>
-      <c r="H19" s="2" t="s">
-        <v>125</v>
-      </c>
       <c r="I19" s="2" t="s">
-        <v>44</v>
+        <v>42</v>
       </c>
       <c r="J19" s="3" t="s">
         <v>13</v>
@@ -3382,159 +3359,159 @@
     </row>
     <row r="20" ht="48" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A20" s="2" t="s">
+        <v>279</v>
+      </c>
+      <c r="B20" s="2" t="s">
+        <v>280</v>
+      </c>
+      <c r="C20" s="2" t="s">
+        <v>281</v>
+      </c>
+      <c r="D20" s="2" t="s">
+        <v>188</v>
+      </c>
+      <c r="E20" s="2" t="s">
         <v>282</v>
       </c>
-      <c r="B20" s="2" t="s">
+      <c r="F20" s="2" t="s">
         <v>283</v>
       </c>
-      <c r="C20" s="2" t="s">
+      <c r="G20" s="2" t="s">
         <v>284</v>
       </c>
-      <c r="D20" s="2" t="s">
-        <v>191</v>
-      </c>
-      <c r="E20" s="2" t="s">
-        <v>285</v>
-      </c>
-      <c r="F20" s="2" t="s">
-        <v>286</v>
-      </c>
-      <c r="G20" s="2" t="s">
-        <v>287</v>
-      </c>
       <c r="H20" s="2" t="s">
-        <v>90</v>
+        <v>88</v>
       </c>
       <c r="I20" s="2" t="s">
-        <v>109</v>
-      </c>
-      <c r="J20" s="6" t="s">
+        <v>107</v>
+      </c>
+      <c r="J20" s="5" t="s">
         <v>4</v>
       </c>
     </row>
     <row r="21" ht="48" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A21" s="2" t="s">
+        <v>285</v>
+      </c>
+      <c r="B21" s="2" t="s">
+        <v>280</v>
+      </c>
+      <c r="C21" s="2" t="s">
+        <v>286</v>
+      </c>
+      <c r="D21" s="2" t="s">
+        <v>188</v>
+      </c>
+      <c r="E21" s="2" t="s">
+        <v>287</v>
+      </c>
+      <c r="F21" s="2" t="s">
         <v>288</v>
       </c>
-      <c r="B21" s="2" t="s">
-        <v>283</v>
-      </c>
-      <c r="C21" s="2" t="s">
+      <c r="G21" s="2" t="s">
         <v>289</v>
       </c>
-      <c r="D21" s="2" t="s">
-        <v>191</v>
-      </c>
-      <c r="E21" s="2" t="s">
-        <v>290</v>
-      </c>
-      <c r="F21" s="2" t="s">
-        <v>291</v>
-      </c>
-      <c r="G21" s="2" t="s">
-        <v>292</v>
-      </c>
       <c r="H21" s="2" t="s">
-        <v>90</v>
+        <v>88</v>
       </c>
       <c r="I21" s="2" t="s">
-        <v>109</v>
-      </c>
-      <c r="J21" s="6" t="s">
+        <v>107</v>
+      </c>
+      <c r="J21" s="5" t="s">
         <v>4</v>
       </c>
     </row>
     <row r="22" ht="48" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A22" s="2" t="s">
+        <v>290</v>
+      </c>
+      <c r="B22" s="2" t="s">
+        <v>280</v>
+      </c>
+      <c r="C22" s="2" t="s">
+        <v>291</v>
+      </c>
+      <c r="D22" s="2" t="s">
+        <v>188</v>
+      </c>
+      <c r="E22" s="2" t="s">
+        <v>292</v>
+      </c>
+      <c r="F22" s="2" t="s">
         <v>293</v>
       </c>
-      <c r="B22" s="2" t="s">
-        <v>283</v>
-      </c>
-      <c r="C22" s="2" t="s">
+      <c r="G22" s="2" t="s">
         <v>294</v>
       </c>
-      <c r="D22" s="2" t="s">
-        <v>191</v>
-      </c>
-      <c r="E22" s="2" t="s">
-        <v>295</v>
-      </c>
-      <c r="F22" s="2" t="s">
-        <v>296</v>
-      </c>
-      <c r="G22" s="2" t="s">
-        <v>297</v>
-      </c>
       <c r="H22" s="2" t="s">
-        <v>90</v>
+        <v>88</v>
       </c>
       <c r="I22" s="2" t="s">
-        <v>109</v>
-      </c>
-      <c r="J22" s="6" t="s">
+        <v>107</v>
+      </c>
+      <c r="J22" s="5" t="s">
         <v>4</v>
       </c>
     </row>
     <row r="23" ht="48" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A23" s="2" t="s">
+        <v>295</v>
+      </c>
+      <c r="B23" s="2" t="s">
+        <v>280</v>
+      </c>
+      <c r="C23" s="2" t="s">
+        <v>296</v>
+      </c>
+      <c r="D23" s="2" t="s">
+        <v>297</v>
+      </c>
+      <c r="E23" s="2" t="s">
         <v>298</v>
       </c>
-      <c r="B23" s="2" t="s">
-        <v>283</v>
-      </c>
-      <c r="C23" s="2" t="s">
+      <c r="F23" s="2" t="s">
         <v>299</v>
       </c>
-      <c r="D23" s="2" t="s">
+      <c r="G23" s="2" t="s">
         <v>300</v>
       </c>
-      <c r="E23" s="2" t="s">
+      <c r="H23" s="2" t="s">
         <v>301</v>
       </c>
-      <c r="F23" s="2" t="s">
-        <v>302</v>
-      </c>
-      <c r="G23" s="2" t="s">
-        <v>303</v>
-      </c>
-      <c r="H23" s="2" t="s">
-        <v>304</v>
-      </c>
       <c r="I23" s="2" t="s">
-        <v>109</v>
-      </c>
-      <c r="J23" s="6" t="s">
+        <v>107</v>
+      </c>
+      <c r="J23" s="5" t="s">
         <v>4</v>
       </c>
     </row>
     <row r="24" ht="48" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A24" s="2" t="s">
+        <v>302</v>
+      </c>
+      <c r="B24" s="2" t="s">
+        <v>303</v>
+      </c>
+      <c r="C24" s="2" t="s">
+        <v>304</v>
+      </c>
+      <c r="D24" s="2" t="s">
+        <v>232</v>
+      </c>
+      <c r="E24" s="2" t="s">
         <v>305</v>
       </c>
-      <c r="B24" s="2" t="s">
+      <c r="F24" s="2" t="s">
+        <v>88</v>
+      </c>
+      <c r="G24" s="2" t="s">
         <v>306</v>
       </c>
-      <c r="C24" s="2" t="s">
-        <v>307</v>
-      </c>
-      <c r="D24" s="2" t="s">
-        <v>235</v>
-      </c>
-      <c r="E24" s="2" t="s">
-        <v>308</v>
-      </c>
-      <c r="F24" s="2" t="s">
-        <v>90</v>
-      </c>
-      <c r="G24" s="2" t="s">
-        <v>309</v>
-      </c>
       <c r="H24" s="2" t="s">
-        <v>90</v>
+        <v>88</v>
       </c>
       <c r="I24" s="2" t="s">
-        <v>44</v>
+        <v>42</v>
       </c>
       <c r="J24" s="3" t="s">
         <v>13</v>
@@ -3542,97 +3519,97 @@
     </row>
     <row r="25" ht="48" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A25" s="2" t="s">
+        <v>307</v>
+      </c>
+      <c r="B25" s="2" t="s">
+        <v>303</v>
+      </c>
+      <c r="C25" s="2" t="s">
+        <v>308</v>
+      </c>
+      <c r="D25" s="2" t="s">
+        <v>188</v>
+      </c>
+      <c r="E25" s="2" t="s">
+        <v>309</v>
+      </c>
+      <c r="F25" s="2" t="s">
+        <v>88</v>
+      </c>
+      <c r="G25" s="2" t="s">
         <v>310</v>
       </c>
-      <c r="B25" s="2" t="s">
-        <v>306</v>
-      </c>
-      <c r="C25" s="2" t="s">
-        <v>311</v>
-      </c>
-      <c r="D25" s="2" t="s">
-        <v>191</v>
-      </c>
-      <c r="E25" s="2" t="s">
-        <v>312</v>
-      </c>
-      <c r="F25" s="2" t="s">
-        <v>90</v>
-      </c>
-      <c r="G25" s="2" t="s">
-        <v>313</v>
-      </c>
       <c r="H25" s="2" t="s">
-        <v>90</v>
+        <v>88</v>
       </c>
       <c r="I25" s="2" t="s">
-        <v>109</v>
-      </c>
-      <c r="J25" s="6" t="s">
+        <v>107</v>
+      </c>
+      <c r="J25" s="5" t="s">
         <v>4</v>
       </c>
     </row>
     <row r="26" ht="48" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A26" s="2" t="s">
+        <v>311</v>
+      </c>
+      <c r="B26" s="2" t="s">
+        <v>303</v>
+      </c>
+      <c r="C26" s="2" t="s">
+        <v>312</v>
+      </c>
+      <c r="D26" s="2" t="s">
+        <v>188</v>
+      </c>
+      <c r="E26" s="2" t="s">
+        <v>313</v>
+      </c>
+      <c r="F26" s="2" t="s">
         <v>314</v>
       </c>
-      <c r="B26" s="2" t="s">
-        <v>306</v>
-      </c>
-      <c r="C26" s="2" t="s">
+      <c r="G26" s="2" t="s">
         <v>315</v>
       </c>
-      <c r="D26" s="2" t="s">
-        <v>191</v>
-      </c>
-      <c r="E26" s="2" t="s">
-        <v>316</v>
-      </c>
-      <c r="F26" s="2" t="s">
-        <v>317</v>
-      </c>
-      <c r="G26" s="2" t="s">
-        <v>318</v>
-      </c>
       <c r="H26" s="2" t="s">
-        <v>90</v>
+        <v>88</v>
       </c>
       <c r="I26" s="2" t="s">
-        <v>109</v>
-      </c>
-      <c r="J26" s="6" t="s">
+        <v>107</v>
+      </c>
+      <c r="J26" s="5" t="s">
         <v>4</v>
       </c>
     </row>
     <row r="27" ht="48" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A27" s="2" t="s">
+        <v>316</v>
+      </c>
+      <c r="B27" s="2" t="s">
+        <v>303</v>
+      </c>
+      <c r="C27" s="2" t="s">
+        <v>317</v>
+      </c>
+      <c r="D27" s="2" t="s">
+        <v>318</v>
+      </c>
+      <c r="E27" s="2" t="s">
         <v>319</v>
       </c>
-      <c r="B27" s="2" t="s">
-        <v>306</v>
-      </c>
-      <c r="C27" s="2" t="s">
+      <c r="F27" s="2" t="s">
         <v>320</v>
       </c>
-      <c r="D27" s="2" t="s">
+      <c r="G27" s="2" t="s">
         <v>321</v>
       </c>
-      <c r="E27" s="2" t="s">
+      <c r="H27" s="2" t="s">
         <v>322</v>
       </c>
-      <c r="F27" s="2" t="s">
-        <v>323</v>
-      </c>
-      <c r="G27" s="2" t="s">
-        <v>324</v>
-      </c>
-      <c r="H27" s="2" t="s">
-        <v>325</v>
-      </c>
       <c r="I27" s="2" t="s">
-        <v>109</v>
-      </c>
-      <c r="J27" s="6" t="s">
+        <v>107</v>
+      </c>
+      <c r="J27" s="5" t="s">
         <v>4</v>
       </c>
     </row>
@@ -3661,63 +3638,63 @@
   <sheetData>
     <row r="1" ht="28" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
+        <v>24</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>25</v>
+      </c>
+      <c r="C1" s="1" t="s">
         <v>26</v>
       </c>
-      <c r="B1" s="1" t="s">
+      <c r="D1" s="1" t="s">
         <v>27</v>
       </c>
-      <c r="C1" s="1" t="s">
+      <c r="E1" s="1" t="s">
         <v>28</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="F1" s="1" t="s">
         <v>29</v>
       </c>
-      <c r="E1" s="1" t="s">
+      <c r="G1" s="1" t="s">
         <v>30</v>
       </c>
-      <c r="F1" s="1" t="s">
+      <c r="H1" s="1" t="s">
         <v>31</v>
       </c>
-      <c r="G1" s="1" t="s">
+      <c r="I1" s="1" t="s">
         <v>32</v>
       </c>
-      <c r="H1" s="1" t="s">
+      <c r="J1" s="1" t="s">
         <v>33</v>
-      </c>
-      <c r="I1" s="1" t="s">
-        <v>34</v>
-      </c>
-      <c r="J1" s="1" t="s">
-        <v>35</v>
       </c>
     </row>
     <row r="2" ht="64" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A2" s="2" t="s">
+        <v>323</v>
+      </c>
+      <c r="B2" s="2" t="s">
+        <v>324</v>
+      </c>
+      <c r="C2" s="2" t="s">
+        <v>325</v>
+      </c>
+      <c r="D2" s="2" t="s">
         <v>326</v>
       </c>
-      <c r="B2" s="2" t="s">
+      <c r="E2" s="2" t="s">
         <v>327</v>
       </c>
-      <c r="C2" s="2" t="s">
+      <c r="F2" s="2" t="s">
+        <v>39</v>
+      </c>
+      <c r="G2" s="2" t="s">
         <v>328</v>
       </c>
-      <c r="D2" s="2" t="s">
+      <c r="H2" s="2" t="s">
         <v>329</v>
       </c>
-      <c r="E2" s="2" t="s">
-        <v>330</v>
-      </c>
-      <c r="F2" s="2" t="s">
-        <v>41</v>
-      </c>
-      <c r="G2" s="2" t="s">
-        <v>331</v>
-      </c>
-      <c r="H2" s="2" t="s">
-        <v>332</v>
-      </c>
       <c r="I2" s="2" t="s">
-        <v>44</v>
+        <v>42</v>
       </c>
       <c r="J2" s="3" t="s">
         <v>13</v>
@@ -3725,31 +3702,31 @@
     </row>
     <row r="3" ht="48" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A3" s="2" t="s">
+        <v>330</v>
+      </c>
+      <c r="B3" s="2" t="s">
+        <v>331</v>
+      </c>
+      <c r="C3" s="2" t="s">
+        <v>332</v>
+      </c>
+      <c r="D3" s="2" t="s">
         <v>333</v>
       </c>
-      <c r="B3" s="2" t="s">
+      <c r="E3" s="2" t="s">
         <v>334</v>
       </c>
-      <c r="C3" s="2" t="s">
+      <c r="F3" s="2" t="s">
+        <v>39</v>
+      </c>
+      <c r="G3" s="2" t="s">
         <v>335</v>
       </c>
-      <c r="D3" s="2" t="s">
+      <c r="H3" s="2" t="s">
         <v>336</v>
       </c>
-      <c r="E3" s="2" t="s">
-        <v>337</v>
-      </c>
-      <c r="F3" s="2" t="s">
-        <v>41</v>
-      </c>
-      <c r="G3" s="2" t="s">
-        <v>338</v>
-      </c>
-      <c r="H3" s="2" t="s">
-        <v>339</v>
-      </c>
       <c r="I3" s="2" t="s">
-        <v>44</v>
+        <v>42</v>
       </c>
       <c r="J3" s="3" t="s">
         <v>13</v>
@@ -3757,31 +3734,31 @@
     </row>
     <row r="4" ht="48" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A4" s="2" t="s">
+        <v>337</v>
+      </c>
+      <c r="B4" s="2" t="s">
+        <v>338</v>
+      </c>
+      <c r="C4" s="2" t="s">
+        <v>339</v>
+      </c>
+      <c r="D4" s="2" t="s">
         <v>340</v>
       </c>
-      <c r="B4" s="2" t="s">
+      <c r="E4" s="2" t="s">
         <v>341</v>
       </c>
-      <c r="C4" s="2" t="s">
+      <c r="F4" s="2" t="s">
         <v>342</v>
       </c>
-      <c r="D4" s="2" t="s">
+      <c r="G4" s="2" t="s">
         <v>343</v>
       </c>
-      <c r="E4" s="2" t="s">
+      <c r="H4" s="2" t="s">
         <v>344</v>
       </c>
-      <c r="F4" s="2" t="s">
-        <v>345</v>
-      </c>
-      <c r="G4" s="2" t="s">
-        <v>346</v>
-      </c>
-      <c r="H4" s="2" t="s">
-        <v>347</v>
-      </c>
       <c r="I4" s="2" t="s">
-        <v>44</v>
+        <v>42</v>
       </c>
       <c r="J4" s="3" t="s">
         <v>13</v>
@@ -3812,63 +3789,63 @@
   <sheetData>
     <row r="1" ht="28" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
+        <v>24</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>25</v>
+      </c>
+      <c r="C1" s="1" t="s">
         <v>26</v>
       </c>
-      <c r="B1" s="1" t="s">
+      <c r="D1" s="1" t="s">
         <v>27</v>
       </c>
-      <c r="C1" s="1" t="s">
+      <c r="E1" s="1" t="s">
         <v>28</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="F1" s="1" t="s">
         <v>29</v>
       </c>
-      <c r="E1" s="1" t="s">
+      <c r="G1" s="1" t="s">
         <v>30</v>
       </c>
-      <c r="F1" s="1" t="s">
+      <c r="H1" s="1" t="s">
         <v>31</v>
       </c>
-      <c r="G1" s="1" t="s">
+      <c r="I1" s="1" t="s">
         <v>32</v>
       </c>
-      <c r="H1" s="1" t="s">
+      <c r="J1" s="1" t="s">
         <v>33</v>
-      </c>
-      <c r="I1" s="1" t="s">
-        <v>34</v>
-      </c>
-      <c r="J1" s="1" t="s">
-        <v>35</v>
       </c>
     </row>
     <row r="2" ht="64" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A2" s="2" t="s">
-        <v>348</v>
+        <v>345</v>
       </c>
       <c r="B2" s="2" t="s">
+        <v>324</v>
+      </c>
+      <c r="C2" s="2" t="s">
+        <v>325</v>
+      </c>
+      <c r="D2" s="2" t="s">
+        <v>326</v>
+      </c>
+      <c r="E2" s="2" t="s">
         <v>327</v>
       </c>
-      <c r="C2" s="2" t="s">
+      <c r="F2" s="2" t="s">
+        <v>39</v>
+      </c>
+      <c r="G2" s="2" t="s">
         <v>328</v>
       </c>
-      <c r="D2" s="2" t="s">
+      <c r="H2" s="2" t="s">
         <v>329</v>
       </c>
-      <c r="E2" s="2" t="s">
-        <v>330</v>
-      </c>
-      <c r="F2" s="2" t="s">
-        <v>41</v>
-      </c>
-      <c r="G2" s="2" t="s">
-        <v>331</v>
-      </c>
-      <c r="H2" s="2" t="s">
-        <v>332</v>
-      </c>
       <c r="I2" s="2" t="s">
-        <v>44</v>
+        <v>42</v>
       </c>
       <c r="J2" s="3" t="s">
         <v>13</v>
@@ -3876,31 +3853,31 @@
     </row>
     <row r="3" ht="48" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A3" s="2" t="s">
-        <v>349</v>
+        <v>346</v>
       </c>
       <c r="B3" s="2" t="s">
+        <v>331</v>
+      </c>
+      <c r="C3" s="2" t="s">
+        <v>332</v>
+      </c>
+      <c r="D3" s="2" t="s">
+        <v>333</v>
+      </c>
+      <c r="E3" s="2" t="s">
         <v>334</v>
       </c>
-      <c r="C3" s="2" t="s">
+      <c r="F3" s="2" t="s">
+        <v>39</v>
+      </c>
+      <c r="G3" s="2" t="s">
         <v>335</v>
       </c>
-      <c r="D3" s="2" t="s">
+      <c r="H3" s="2" t="s">
         <v>336</v>
       </c>
-      <c r="E3" s="2" t="s">
-        <v>337</v>
-      </c>
-      <c r="F3" s="2" t="s">
-        <v>41</v>
-      </c>
-      <c r="G3" s="2" t="s">
-        <v>338</v>
-      </c>
-      <c r="H3" s="2" t="s">
-        <v>339</v>
-      </c>
       <c r="I3" s="2" t="s">
-        <v>44</v>
+        <v>42</v>
       </c>
       <c r="J3" s="3" t="s">
         <v>13</v>
@@ -3908,31 +3885,31 @@
     </row>
     <row r="4" ht="48" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A4" s="2" t="s">
-        <v>350</v>
+        <v>347</v>
       </c>
       <c r="B4" s="2" t="s">
+        <v>338</v>
+      </c>
+      <c r="C4" s="2" t="s">
+        <v>339</v>
+      </c>
+      <c r="D4" s="2" t="s">
+        <v>340</v>
+      </c>
+      <c r="E4" s="2" t="s">
         <v>341</v>
       </c>
-      <c r="C4" s="2" t="s">
+      <c r="F4" s="2" t="s">
         <v>342</v>
       </c>
-      <c r="D4" s="2" t="s">
+      <c r="G4" s="2" t="s">
         <v>343</v>
       </c>
-      <c r="E4" s="2" t="s">
-        <v>344</v>
-      </c>
-      <c r="F4" s="2" t="s">
-        <v>345</v>
-      </c>
-      <c r="G4" s="2" t="s">
-        <v>346</v>
-      </c>
       <c r="H4" s="2" t="s">
-        <v>351</v>
+        <v>348</v>
       </c>
       <c r="I4" s="2" t="s">
-        <v>44</v>
+        <v>42</v>
       </c>
       <c r="J4" s="3" t="s">
         <v>13</v>
@@ -3940,31 +3917,31 @@
     </row>
     <row r="5" ht="64" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A5" s="2" t="s">
+        <v>349</v>
+      </c>
+      <c r="B5" s="2" t="s">
+        <v>350</v>
+      </c>
+      <c r="C5" s="2" t="s">
+        <v>351</v>
+      </c>
+      <c r="D5" s="2" t="s">
         <v>352</v>
       </c>
-      <c r="B5" s="2" t="s">
+      <c r="E5" s="2" t="s">
         <v>353</v>
       </c>
-      <c r="C5" s="2" t="s">
+      <c r="F5" s="2" t="s">
         <v>354</v>
       </c>
-      <c r="D5" s="2" t="s">
+      <c r="G5" s="2" t="s">
         <v>355</v>
       </c>
-      <c r="E5" s="2" t="s">
+      <c r="H5" s="2" t="s">
         <v>356</v>
       </c>
-      <c r="F5" s="2" t="s">
-        <v>357</v>
-      </c>
-      <c r="G5" s="2" t="s">
-        <v>358</v>
-      </c>
-      <c r="H5" s="2" t="s">
-        <v>359</v>
-      </c>
       <c r="I5" s="2" t="s">
-        <v>44</v>
+        <v>42</v>
       </c>
       <c r="J5" s="3" t="s">
         <v>13</v>

</xml_diff>